<commit_message>
Align current demo flow and fixture data
</commit_message>
<xml_diff>
--- a/public/demo-data/TRK-DEMO-001/input/Cargo_Details_TRK-DEMO-001.xlsx
+++ b/public/demo-data/TRK-DEMO-001/input/Cargo_Details_TRK-DEMO-001.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cargo Details" sheetId="1" r:id="Rc65746cb8c4c4cd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cargo Details" sheetId="1" r:id="R03f85a4f3cce47d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -45,8 +45,25 @@
       <x:color rgb="FF4B5563"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17242E"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF17242E"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF63717C"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -66,6 +83,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF123A63"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7E8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -89,7 +121,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -136,6 +168,41 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -338,139 +405,208 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="8.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="9.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="23.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="9.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="11.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="8" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="9.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="8.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="8" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="33" customHeight="1">
+      <x:c r="A1" s="20" t="str">
         <x:v>Cargo Details TRK-DEMO-001</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-      <x:c r="K1" s="3"/>
-      <x:c r="L1" s="3"/>
-      <x:c r="M1" s="3"/>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
+      <x:c r="I1" s="20"/>
+      <x:c r="J1" s="20"/>
+      <x:c r="K1" s="20"/>
+      <x:c r="L1" s="20"/>
+      <x:c r="M1" s="20"/>
+      <x:c r="N1" s="20"/>
     </x:row>
-    <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+    <x:row r="2" ht="37.5" customHeight="1">
+      <x:c r="A2" s="26" t="str">
         <x:v>Line ID</x:v>
       </x:c>
-      <x:c r="B2" s="8" t="str">
+      <x:c r="B2" s="26" t="str">
+        <x:v>Delivery Stop ID</x:v>
+      </x:c>
+      <x:c r="C2" s="26" t="str">
         <x:v>H/U Type</x:v>
       </x:c>
-      <x:c r="C2" s="8" t="str">
+      <x:c r="D2" s="26" t="str">
         <x:v>H/U Count</x:v>
       </x:c>
-      <x:c r="D2" s="8" t="str">
+      <x:c r="E2" s="26" t="str">
         <x:v>Package Type</x:v>
       </x:c>
-      <x:c r="E2" s="8" t="str">
+      <x:c r="F2" s="26" t="str">
         <x:v>Piece Count</x:v>
       </x:c>
-      <x:c r="F2" s="8" t="str">
+      <x:c r="G2" s="26" t="str">
         <x:v>Commodity Description</x:v>
       </x:c>
-      <x:c r="G2" s="8" t="str">
+      <x:c r="H2" s="26" t="str">
         <x:v>Total Weight (lb)</x:v>
       </x:c>
-      <x:c r="H2" s="8" t="str">
+      <x:c r="I2" s="26" t="str">
         <x:v>Dimensions (in)</x:v>
       </x:c>
-      <x:c r="I2" s="8" t="str">
+      <x:c r="J2" s="26" t="str">
         <x:v>Freight Class</x:v>
       </x:c>
-      <x:c r="J2" s="8" t="str">
+      <x:c r="K2" s="26" t="str">
         <x:v>NMFC</x:v>
       </x:c>
-      <x:c r="K2" s="8" t="str">
+      <x:c r="L2" s="26" t="str">
         <x:v>Stackable</x:v>
       </x:c>
-      <x:c r="L2" s="8" t="str">
+      <x:c r="M2" s="26" t="str">
         <x:v>Turnable</x:v>
       </x:c>
-      <x:c r="M2" s="8" t="str">
+      <x:c r="N2" s="26" t="str">
         <x:v>Hazmat</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="10" t="str">
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="29" t="str">
         <x:v>CARGO-001</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
+      <x:c r="B3" s="29" t="str">
+        <x:v>STOP-DEMO-002</x:v>
+      </x:c>
+      <x:c r="C3" s="29" t="str">
         <x:v>Pallet</x:v>
       </x:c>
-      <x:c r="C3" s="13" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D3" s="10" t="str">
+      <x:c r="D3" s="30" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E3" s="29" t="str">
         <x:v>Carton</x:v>
       </x:c>
-      <x:c r="E3" s="13" t="n">
+      <x:c r="F3" s="30" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F3" s="10" t="str">
+      <x:c r="G3" s="29" t="str">
         <x:v>Consumer electronic accessories</x:v>
       </x:c>
-      <x:c r="G3" s="14" t="n">
+      <x:c r="H3" s="30" t="n">
         <x:v>2450</x:v>
       </x:c>
-      <x:c r="H3" s="10" t="str">
+      <x:c r="I3" s="29" t="str">
         <x:v>48 x 40 x 48</x:v>
       </x:c>
-      <x:c r="I3" s="15" t="str">
+      <x:c r="J3" s="29" t="str">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="J3" s="15" t="str"/>
-      <x:c r="K3" s="15" t="str">
+      <x:c r="K3" s="29" t="str"/>
+      <x:c r="L3" s="29" t="str">
         <x:v>Yes</x:v>
       </x:c>
-      <x:c r="L3" s="15" t="str">
-        <x:v>Not confirmed</x:v>
-      </x:c>
-      <x:c r="M3" s="15" t="str">
+      <x:c r="M3" s="29" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="N3" s="29" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="17" t="str">
-        <x:v>Shipment total: 10 pallets, 120 cartons, 2,450 lb. Turnable status requires Operations confirmation.</x:v>
-      </x:c>
-      <x:c r="B5" s="17"/>
-      <x:c r="C5" s="17"/>
-      <x:c r="D5" s="17"/>
-      <x:c r="E5" s="17"/>
-      <x:c r="F5" s="17"/>
-      <x:c r="G5" s="17"/>
-      <x:c r="H5" s="17"/>
-      <x:c r="I5" s="17"/>
-      <x:c r="J5" s="17"/>
-      <x:c r="K5" s="17"/>
-      <x:c r="L5" s="17"/>
-      <x:c r="M5" s="17"/>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="28" t="str">
+        <x:v>CARGO-002</x:v>
+      </x:c>
+      <x:c r="B4" s="28" t="str">
+        <x:v>STOP-DEMO-003</x:v>
+      </x:c>
+      <x:c r="C4" s="28" t="str">
+        <x:v>Pallet</x:v>
+      </x:c>
+      <x:c r="D4" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E4" s="28" t="str">
+        <x:v>Carton</x:v>
+      </x:c>
+      <x:c r="F4" s="31" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G4" s="28" t="str">
+        <x:v>Medical device accessories</x:v>
+      </x:c>
+      <x:c r="H4" s="31" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="I4" s="28" t="str">
+        <x:v>48 x 40 x 42</x:v>
+      </x:c>
+      <x:c r="J4" s="28" t="str">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="K4" s="28" t="str">
+        <x:v>184140</x:v>
+      </x:c>
+      <x:c r="L4" s="28" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="M4" s="28" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N4" s="28" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="9" customHeight="1">
+      <x:c r="A5" s="18"/>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="18"/>
+      <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18"/>
+      <x:c r="G5" s="18"/>
+      <x:c r="H5" s="18"/>
+      <x:c r="I5" s="18"/>
+      <x:c r="J5" s="18"/>
+      <x:c r="K5" s="18"/>
+      <x:c r="L5" s="18"/>
+      <x:c r="M5" s="18"/>
+      <x:c r="N5" s="18"/>
+    </x:row>
+    <x:row r="6" ht="25.5" customHeight="1">
+      <x:c r="A6" s="34" t="str">
+        <x:v>Shipment total: 12 pallets, 168 cartons, 3,950 lb. Cargo is allocated to two delivery stops.</x:v>
+      </x:c>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="34"/>
+      <x:c r="D6" s="34"/>
+      <x:c r="E6" s="34"/>
+      <x:c r="F6" s="34"/>
+      <x:c r="G6" s="34"/>
+      <x:c r="H6" s="34"/>
+      <x:c r="I6" s="34"/>
+      <x:c r="J6" s="34"/>
+      <x:c r="K6" s="34"/>
+      <x:c r="L6" s="34"/>
+      <x:c r="M6" s="34"/>
+      <x:c r="N6" s="34"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A5:M5"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A6:N6"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>